<commit_message>
use tenacity and implementation for LSI and fix for no GSI and LSI
</commit_message>
<xml_diff>
--- a/input_specification_files/CUSTOMER_POLICY.xlsx
+++ b/input_specification_files/CUSTOMER_POLICY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chethgan/Desktop/TFC/DAL_PROMPT_GENERATOR/input_specification_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144E3D57-77D1-164C-8A87-16584EDD01F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D249FE03-3822-EE4B-ABFD-24170E445624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{E6005EB9-FFA4-4870-9B6D-5690CA9B2A4B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17460" xr2:uid="{E6005EB9-FFA4-4870-9B6D-5690CA9B2A4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="60">
   <si>
     <t>TABLE_NAME</t>
   </si>
@@ -202,6 +202,21 @@
   </si>
   <si>
     <t>(policy_name risk_id address premium sum_insured policy_version start_date end_date),(keys~projected)</t>
+  </si>
+  <si>
+    <t>LSI_SKs</t>
+  </si>
+  <si>
+    <t>LSI_PROJECTIONs</t>
+  </si>
+  <si>
+    <t>Lsi sort key (optional). Comma seperated</t>
+  </si>
+  <si>
+    <t>column_lsi_sk_1,column_lsi_sk_2,column_lsi_sk_3,column_lsi_sk_4</t>
+  </si>
+  <si>
+    <t>Lsi projections (optional). Comma seperated.~ to be used for key projected and all attributes projected instead of space</t>
   </si>
 </sst>
 </file>
@@ -573,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826647F6-C730-4829-AD38-A94D4D230085}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -585,12 +600,14 @@
     <col min="7" max="7" width="43.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="81.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" customWidth="1"/>
+    <col min="12" max="12" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -619,16 +636,22 @@
         <v>36</v>
       </c>
       <c r="J1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -656,17 +679,17 @@
       <c r="I2" t="s">
         <v>53</v>
       </c>
-      <c r="J2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" t="s">
-        <v>7</v>
-      </c>
       <c r="L2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -694,13 +717,13 @@
       <c r="I3" t="s">
         <v>54</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>7</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>7</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -713,7 +736,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{603EC8F7-6F1C-4FD2-BCF2-C2570A90EA43}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
@@ -833,34 +856,56 @@
     </row>
     <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>